<commit_message>
added Environment setup and DriverFactory classes
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/testData1.xlsx
+++ b/src/test/resources/testdata/testData1.xlsx
@@ -4,20 +4,21 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="4" rupBuild="9302"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2430" windowWidth="13020" windowHeight="5940" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="2430" windowWidth="13020" windowHeight="5940" activeTab="4"/>
   </bookViews>
   <sheets>
-    <sheet name="ValidData" sheetId="1" r:id="rId1"/>
+    <sheet name="ValidLoginLocal" sheetId="1" r:id="rId1"/>
     <sheet name="InvalidData" sheetId="2" r:id="rId2"/>
     <sheet name="empDetails" sheetId="3" r:id="rId3"/>
+    <sheet name="ValidLoginRemote" sheetId="4" r:id="rId4"/>
+    <sheet name="CreateEmpDetails" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="0"/>
-  <oleSize ref="A1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="30">
   <si>
     <t>userName</t>
   </si>
@@ -62,6 +63,51 @@
   </si>
   <si>
     <t>deepak</t>
+  </si>
+  <si>
+    <t>Admin</t>
+  </si>
+  <si>
+    <t>admin123</t>
+  </si>
+  <si>
+    <t>Fname</t>
+  </si>
+  <si>
+    <t>Mname</t>
+  </si>
+  <si>
+    <t>Lname</t>
+  </si>
+  <si>
+    <t>Eid</t>
+  </si>
+  <si>
+    <t>username</t>
+  </si>
+  <si>
+    <t>pass</t>
+  </si>
+  <si>
+    <t>conPass</t>
+  </si>
+  <si>
+    <t>Manish</t>
+  </si>
+  <si>
+    <t>Kumar</t>
+  </si>
+  <si>
+    <t>Man123456</t>
+  </si>
+  <si>
+    <t>pic</t>
+  </si>
+  <si>
+    <t>D:\manish work space\eclipse setup\orangehrm_automation\src\test\resources\testdata\samplePic.jpg</t>
+  </si>
+  <si>
+    <t>manishKumar</t>
   </si>
 </sst>
 </file>
@@ -528,4 +574,95 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B2" r:id="rId1" display="Manish@880"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D2">
+        <v>104261</v>
+      </c>
+      <c r="E2" t="s">
+        <v>29</v>
+      </c>
+      <c r="F2" t="s">
+        <v>26</v>
+      </c>
+      <c r="G2" t="s">
+        <v>26</v>
+      </c>
+      <c r="H2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>